<commit_message>
Another rewrite for adding new tourneys in the future
</commit_message>
<xml_diff>
--- a/output/ukrdl.xlsx
+++ b/output/ukrdl.xlsx
@@ -1,126 +1,54 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
-  <si>
-    <t>Назва</t>
-  </si>
-  <si>
-    <t>ukrDL</t>
-  </si>
-  <si>
-    <t>Олександрійська трилогія. Зима</t>
-  </si>
-  <si>
-    <t>Синхрон ЛУК. Зима</t>
-  </si>
-  <si>
-    <t>Зимовий Major ЛУК</t>
-  </si>
-  <si>
-    <t>Товстолобик</t>
-  </si>
-  <si>
-    <t>Синхрон ЛУК. Весна</t>
-  </si>
-  <si>
-    <t>Minor ЛУК</t>
-  </si>
-  <si>
-    <t>Simply Green</t>
-  </si>
-  <si>
-    <t>Синхрон ЛУК. Літо</t>
-  </si>
-  <si>
-    <t>Літній Major ЛУК</t>
-  </si>
-  <si>
-    <t>Синхрон синів маминої подруги 3</t>
-  </si>
-  <si>
-    <t>Канхвєта очєнь класна. Тузік вкусний</t>
-  </si>
-  <si>
-    <t>Фінал Сезону ЧУ 2024/2025</t>
-  </si>
-  <si>
-    <t>Українська ліга 24/25. Етап 3</t>
-  </si>
-  <si>
-    <t>Українська ліга 24/25. Етап 4</t>
-  </si>
-  <si>
-    <t>Українська ліга 24/25. Етап 5</t>
-  </si>
-  <si>
-    <t>Дзеркало Відкритого Кубку Одеси 2025</t>
-  </si>
-  <si>
-    <t>Забобони Бонобо 2: Шабаш</t>
-  </si>
-  <si>
-    <t>Борисфен 10: Дарниця</t>
-  </si>
-  <si>
-    <t>HDQ. Pictures</t>
-  </si>
-  <si>
-    <t>Бузький Гард-8</t>
-  </si>
-  <si>
-    <t>Кубок Трішки Несередзем'я-2025</t>
-  </si>
-  <si>
-    <t>Бузький Гард-9</t>
-  </si>
-  <si>
-    <t>Борисфен 11: Ірклій</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="204"/>
+      <family val="2"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -143,21 +71,106 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -445,199 +458,253 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Назва</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>ukrDL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Олександрійська трилогія. Зима</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>3.99</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Синхрон ЛУК. Зима</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>2.75</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Зимовий Major ЛУК</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>5.07</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Товстолобик</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>5.98</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Синхрон ЛУК. Весна</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>3.32</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Minor ЛУК</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>3.82</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Simply Green</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>5.09</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Синхрон ЛУК. Літо</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>4.18</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Літній Major ЛУК</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>5.38</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
-      <c r="A11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Синхрон синів маминої подруги 3</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>4.12</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
-      <c r="A12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Канхвєта очєнь класна. Тузік вкусний</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>4.11</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
-      <c r="A13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Фінал Сезону ЧУ 2024/2025</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>5.5</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
-      <c r="A14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Українська ліга 24/25. Етап 3</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
         <v>3.52</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
-      <c r="A15" t="s">
-        <v>15</v>
-      </c>
-      <c r="B15">
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Українська ліга 24/25. Етап 4</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>4.42</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
-      <c r="A16" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16">
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Українська ліга 24/25. Етап 5</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
         <v>3.89</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
-      <c r="A17" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Дзеркало Відкритого Кубку Одеси 2025</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
         <v>3.02</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
-      <c r="A18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18">
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Забобони Бонобо 2: Шабаш</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
         <v>4.3</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
-      <c r="A19" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19">
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Борисфен 10: Дарниця</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
         <v>3.07</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
-      <c r="A20" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20">
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>HDQ. Pictures</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
         <v>2.47</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
-      <c r="A21" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21">
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Бузький Гард-8</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
         <v>4.57</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
-      <c r="A22" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22">
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Кубок Трішки Несередзем'я-2025</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
         <v>5.77</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
-      <c r="A23" t="s">
-        <v>23</v>
-      </c>
-      <c r="B23">
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Бузький Гард-9</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
         <v>3.91</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
-      <c r="A24" t="s">
-        <v>24</v>
-      </c>
-      <c r="B24">
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Борисфен 11: Ірклій</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
         <v>3.57</v>
       </c>
     </row>

</xml_diff>